<commit_message>
feat: complete payroll and payslip system enhancements, Excel sync, and UI cleanups
</commit_message>
<xml_diff>
--- a/data/employee_info.xlsx
+++ b/data/employee_info.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Employee Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Roles" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +49,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -108,7 +109,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -482,16 +483,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="87" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,11 +517,10 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>EMPLOYEE MASTER DIRECTORY</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>EMPLOYEE MASTER DIRECTORY (DATABASE)</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -534,22 +539,47 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Department</t>
+          <t>Monthly Salary (₹)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Monthly Base Salary (INR)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
           <t>Date of Joining</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Date of Leaving</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Bank Name</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Bank A/C No</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>IFSC Code</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>PAN Number</t>
         </is>
       </c>
     </row>
@@ -561,32 +591,33 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Tanmay</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Senior Accountant</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Accounts &amp; Operations</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>65000</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>9285186964</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>2024-04-01</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -596,143 +627,116 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Sarah Smith</t>
+          <t>Tanmay Patel</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Finance Manager</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Accounts &amp; Operations</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>2024-04-01</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>EMP003</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>David Miller</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Junior Auditor</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Accounts &amp; Operations</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>42000</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>2024-04-01</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>EMP004</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Emma Watson</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Payroll Specialist</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Accounts &amp; Operations</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>2024-04-01</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>EMP006</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Robert Brown</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Tax Consultant</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Accounts &amp; Operations</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>75000</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>2024-04-01</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STIFLINK MANAGEMENT (OPC) PVT. LTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>OFFICE NO. 301 FIFTH FLOOR, ADHARHSILA COMPLEX, GANDHI MAIDAN, PATNA, BIHAR 800001.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>COMPANY ROLES &amp; FIXED SALARY STRUCTURE (DATABASE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Role ID</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Role Title / Designation</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Monthly Base Salary (₹)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ROLE001</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>